<commit_message>
feat: add UAT test cases documentation spreadsheet
</commit_message>
<xml_diff>
--- a/plans/uat-test-cases.xlsx
+++ b/plans/uat-test-cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\gaap\plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{474D93ED-36F3-4329-BF79-5542AC96E5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CB4DDC-2435-40EB-86C5-6A7166AB2A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="uat-test-cases" sheetId="1" r:id="rId1"/>
     <sheet name="资金流水测试" sheetId="2" r:id="rId2"/>
     <sheet name="bug记录" sheetId="3" r:id="rId3"/>
+    <sheet name="TODO" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1109" uniqueCount="695">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="700">
   <si>
     <t>用例编号</t>
   </si>
@@ -2131,6 +2132,37 @@
       </rPr>
       <t xml:space="preserve"> CNY</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>汇率更新时弹窗弹了</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>2次</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>新增账户时，币种使用账户基准货币（注意父子账户也是这个逻辑）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>新增账户时，弹窗弹了多次</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>父账号总资产未使用基准货币，符号不正确</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>已修正</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2247,7 +2279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2257,6 +2289,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2340,6 +2373,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>609195</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="图片 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDB36FA8-5D79-6D71-5F45-B4F4D11324B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6334125" y="628650"/>
+          <a:ext cx="609195" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6760,9 +6842,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0945A39-1BCF-450B-B12F-C18314F42358}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="67.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6788,8 +6871,49 @@
         <v>694</v>
       </c>
     </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="8">
+        <v>46125</v>
+      </c>
+      <c r="B3" t="s">
+        <v>698</v>
+      </c>
+      <c r="C3" t="s">
+        <v>699</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA6171EA-8564-45C5-9BCA-C09464C92F7D}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="95" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
+        <v>697</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>